<commit_message>
refactor: add per carrier mode information
enable per carrier min required osnr
enable per carrier penalty
enable per carrier min-max power range

Signed-off-by: JennyLescop <jenny.lescop@orange.com>
Change-Id: Ia522d1e8d25b352cca4138c53ef98b300358bc46
</commit_message>
<xml_diff>
--- a/tests/data/parser/transmission/results_transmission_expected.xlsx
+++ b/tests/data/parser/transmission/results_transmission_expected.xlsx
@@ -375,7 +375,7 @@
         </is>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="198" customHeight="1">
+    <row r="4" s="1" customFormat="1" ht="252" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Transceiver Site_A
@@ -388,6 +388,9 @@
 	- PDL:: 0.00 dB
 	- Latency: 0.0 ms
 	- Actual pch out:: 0.00 dBm
+	- CD penalty: None dB
+	- PMD penalty:: None dB
+	- PDL penalty:: None dB
 </t>
         </is>
       </c>
@@ -432,6 +435,9 @@
 	- PDL:: 0.00 dB
 	- Latency: 0.39 ms
 	- Actual pch out:: 0.00 dBm
+	- CD penalty: None dB
+	- PMD penalty:: None dB
+	- PDL penalty:: None dB
 </t>
         </is>
       </c>

</xml_diff>